<commit_message>
Mapped_executed file is created only. Updates in midway for 21 aug 2026 Friday (not fully done )
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto20aug26_Thurs.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto20aug26_Thurs.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AVITA\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AVITA\projects\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5688"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1096,7 +1096,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:N245"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1178,7 +1177,7 @@
       </c>
       <c r="J2" s="2"/>
       <c r="N2" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B2, $C$2:$C$949, C2, $D$2:$D$949, D2, $E$2:$E$949, E2) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N2:N65" si="0">IF(COUNTIFS( $B$2:$B$949, B2, $C$2:$C$949, C2, $D$2:$D$949, D2, $E$2:$E$949, E2) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -1212,7 +1211,7 @@
       </c>
       <c r="J3" s="2"/>
       <c r="N3" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B3, $C$2:$C$949, C3, $D$2:$D$949, D3, $E$2:$E$949, E3) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1246,7 +1245,7 @@
       </c>
       <c r="J4" s="2"/>
       <c r="N4" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B4, $C$2:$C$949, C4, $D$2:$D$949, D4, $E$2:$E$949, E4) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1280,7 +1279,7 @@
       </c>
       <c r="J5" s="2"/>
       <c r="N5" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B5, $C$2:$C$949, C5, $D$2:$D$949, D5, $E$2:$E$949, E5) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1314,7 +1313,7 @@
       </c>
       <c r="J6" s="2"/>
       <c r="N6" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B6, $C$2:$C$949, C6, $D$2:$D$949, D6, $E$2:$E$949, E6) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1350,7 +1349,7 @@
         <v>55</v>
       </c>
       <c r="N7" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B7, $C$2:$C$949, C7, $D$2:$D$949, D7, $E$2:$E$949, E7) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1384,7 +1383,7 @@
       </c>
       <c r="J8" s="2"/>
       <c r="N8" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B8, $C$2:$C$949, C8, $D$2:$D$949, D8, $E$2:$E$949, E8) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1423,7 +1422,7 @@
         <v>170</v>
       </c>
       <c r="N9" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B9, $C$2:$C$949, C9, $D$2:$D$949, D9, $E$2:$E$949, E9) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1457,7 +1456,7 @@
       </c>
       <c r="J10" s="2"/>
       <c r="N10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B10, $C$2:$C$949, C10, $D$2:$D$949, D10, $E$2:$E$949, E10) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1493,7 +1492,7 @@
         <v>118</v>
       </c>
       <c r="N11" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B11, $C$2:$C$949, C11, $D$2:$D$949, D11, $E$2:$E$949, E11) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1529,7 +1528,7 @@
         <v>55</v>
       </c>
       <c r="N12" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B12, $C$2:$C$949, C12, $D$2:$D$949, D12, $E$2:$E$949, E12) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1563,7 +1562,7 @@
       </c>
       <c r="J13" s="2"/>
       <c r="N13" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B13, $C$2:$C$949, C13, $D$2:$D$949, D13, $E$2:$E$949, E13) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1597,7 +1596,7 @@
       </c>
       <c r="J14" s="2"/>
       <c r="N14" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B14, $C$2:$C$949, C14, $D$2:$D$949, D14, $E$2:$E$949, E14) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1636,7 +1635,7 @@
         <v>158</v>
       </c>
       <c r="N15" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B15, $C$2:$C$949, C15, $D$2:$D$949, D15, $E$2:$E$949, E15) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1670,7 +1669,7 @@
       </c>
       <c r="J16" s="2"/>
       <c r="N16" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B16, $C$2:$C$949, C16, $D$2:$D$949, D16, $E$2:$E$949, E16) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1706,7 +1705,7 @@
         <v>117</v>
       </c>
       <c r="N17" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B17, $C$2:$C$949, C17, $D$2:$D$949, D17, $E$2:$E$949, E17) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1742,7 +1741,7 @@
         <v>55</v>
       </c>
       <c r="N18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B18, $C$2:$C$949, C18, $D$2:$D$949, D18, $E$2:$E$949, E18) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1776,7 +1775,7 @@
       </c>
       <c r="J19" s="2"/>
       <c r="N19" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B19, $C$2:$C$949, C19, $D$2:$D$949, D19, $E$2:$E$949, E19) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1812,7 +1811,7 @@
         <v>55</v>
       </c>
       <c r="N20" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B20, $C$2:$C$949, C20, $D$2:$D$949, D20, $E$2:$E$949, E20) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1848,7 +1847,7 @@
         <v>41</v>
       </c>
       <c r="N21" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B21, $C$2:$C$949, C21, $D$2:$D$949, D21, $E$2:$E$949, E21) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1882,7 +1881,7 @@
       </c>
       <c r="J22" s="2"/>
       <c r="N22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B22, $C$2:$C$949, C22, $D$2:$D$949, D22, $E$2:$E$949, E22) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1918,7 +1917,7 @@
         <v>55</v>
       </c>
       <c r="N23" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B23, $C$2:$C$949, C23, $D$2:$D$949, D23, $E$2:$E$949, E23) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1952,7 +1951,7 @@
       </c>
       <c r="J24" s="2"/>
       <c r="N24" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B24, $C$2:$C$949, C24, $D$2:$D$949, D24, $E$2:$E$949, E24) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1991,7 +1990,7 @@
         <v>171</v>
       </c>
       <c r="N25" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B25, $C$2:$C$949, C25, $D$2:$D$949, D25, $E$2:$E$949, E25) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2027,7 +2026,7 @@
         <v>41</v>
       </c>
       <c r="N26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B26, $C$2:$C$949, C26, $D$2:$D$949, D26, $E$2:$E$949, E26) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2061,7 +2060,7 @@
       </c>
       <c r="J27" s="2"/>
       <c r="N27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B27, $C$2:$C$949, C27, $D$2:$D$949, D27, $E$2:$E$949, E27) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2097,7 +2096,7 @@
         <v>118</v>
       </c>
       <c r="N28" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B28, $C$2:$C$949, C28, $D$2:$D$949, D28, $E$2:$E$949, E28) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2131,7 +2130,7 @@
       </c>
       <c r="J29" s="2"/>
       <c r="N29" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B29, $C$2:$C$949, C29, $D$2:$D$949, D29, $E$2:$E$949, E29) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2167,7 +2166,7 @@
         <v>55</v>
       </c>
       <c r="N30" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B30, $C$2:$C$949, C30, $D$2:$D$949, D30, $E$2:$E$949, E30) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2201,7 +2200,7 @@
       </c>
       <c r="J31" s="2"/>
       <c r="N31" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B31, $C$2:$C$949, C31, $D$2:$D$949, D31, $E$2:$E$949, E31) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2235,7 +2234,7 @@
       </c>
       <c r="J32" s="2"/>
       <c r="N32" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B32, $C$2:$C$949, C32, $D$2:$D$949, D32, $E$2:$E$949, E32) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2272,7 +2271,7 @@
         <v>146</v>
       </c>
       <c r="N33" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B33, $C$2:$C$949, C33, $D$2:$D$949, D33, $E$2:$E$949, E33) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2306,7 +2305,7 @@
       </c>
       <c r="J34" s="2"/>
       <c r="N34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B34, $C$2:$C$949, C34, $D$2:$D$949, D34, $E$2:$E$949, E34) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2340,7 +2339,7 @@
       </c>
       <c r="J35" s="2"/>
       <c r="N35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B35, $C$2:$C$949, C35, $D$2:$D$949, D35, $E$2:$E$949, E35) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2374,7 +2373,7 @@
       </c>
       <c r="J36" s="2"/>
       <c r="N36" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B36, $C$2:$C$949, C36, $D$2:$D$949, D36, $E$2:$E$949, E36) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2408,7 +2407,7 @@
       </c>
       <c r="J37" s="2"/>
       <c r="N37" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B37, $C$2:$C$949, C37, $D$2:$D$949, D37, $E$2:$E$949, E37) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2444,7 +2443,7 @@
         <v>41</v>
       </c>
       <c r="N38" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B38, $C$2:$C$949, C38, $D$2:$D$949, D38, $E$2:$E$949, E38) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2478,7 +2477,7 @@
       </c>
       <c r="J39" s="2"/>
       <c r="N39" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B39, $C$2:$C$949, C39, $D$2:$D$949, D39, $E$2:$E$949, E39) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2514,7 +2513,7 @@
         <v>117</v>
       </c>
       <c r="N40" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B40, $C$2:$C$949, C40, $D$2:$D$949, D40, $E$2:$E$949, E40) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2548,7 +2547,7 @@
       </c>
       <c r="J41" s="2"/>
       <c r="N41" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B41, $C$2:$C$949, C41, $D$2:$D$949, D41, $E$2:$E$949, E41) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2582,7 +2581,7 @@
       </c>
       <c r="J42" s="2"/>
       <c r="N42" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B42, $C$2:$C$949, C42, $D$2:$D$949, D42, $E$2:$E$949, E42) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2621,7 +2620,7 @@
         <v>170</v>
       </c>
       <c r="N43" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B43, $C$2:$C$949, C43, $D$2:$D$949, D43, $E$2:$E$949, E43) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2655,7 +2654,7 @@
       </c>
       <c r="J44" s="2"/>
       <c r="N44" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B44, $C$2:$C$949, C44, $D$2:$D$949, D44, $E$2:$E$949, E44) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2691,7 +2690,7 @@
         <v>55</v>
       </c>
       <c r="N45" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B45, $C$2:$C$949, C45, $D$2:$D$949, D45, $E$2:$E$949, E45) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2725,7 +2724,7 @@
       </c>
       <c r="J46" s="2"/>
       <c r="N46" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B46, $C$2:$C$949, C46, $D$2:$D$949, D46, $E$2:$E$949, E46) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2759,7 +2758,7 @@
       </c>
       <c r="J47" s="2"/>
       <c r="N47" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B47, $C$2:$C$949, C47, $D$2:$D$949, D47, $E$2:$E$949, E47) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2793,7 +2792,7 @@
       </c>
       <c r="J48" s="2"/>
       <c r="N48" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B48, $C$2:$C$949, C48, $D$2:$D$949, D48, $E$2:$E$949, E48) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2827,7 +2826,7 @@
       </c>
       <c r="J49" s="2"/>
       <c r="N49" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B49, $C$2:$C$949, C49, $D$2:$D$949, D49, $E$2:$E$949, E49) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2863,7 +2862,7 @@
         <v>55</v>
       </c>
       <c r="N50" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B50, $C$2:$C$949, C50, $D$2:$D$949, D50, $E$2:$E$949, E50) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2899,7 +2898,7 @@
         <v>118</v>
       </c>
       <c r="N51" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B51, $C$2:$C$949, C51, $D$2:$D$949, D51, $E$2:$E$949, E51) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2933,7 +2932,7 @@
       </c>
       <c r="J52" s="2"/>
       <c r="N52" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B52, $C$2:$C$949, C52, $D$2:$D$949, D52, $E$2:$E$949, E52) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2967,7 +2966,7 @@
       </c>
       <c r="J53" s="2"/>
       <c r="N53" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B53, $C$2:$C$949, C53, $D$2:$D$949, D53, $E$2:$E$949, E53) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3001,7 +3000,7 @@
       </c>
       <c r="J54" s="2"/>
       <c r="N54" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B54, $C$2:$C$949, C54, $D$2:$D$949, D54, $E$2:$E$949, E54) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3040,7 +3039,7 @@
         <v>171</v>
       </c>
       <c r="N55" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B55, $C$2:$C$949, C55, $D$2:$D$949, D55, $E$2:$E$949, E55) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3074,7 +3073,7 @@
       </c>
       <c r="J56" s="2"/>
       <c r="N56" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B56, $C$2:$C$949, C56, $D$2:$D$949, D56, $E$2:$E$949, E56) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3108,7 +3107,7 @@
       </c>
       <c r="J57" s="2"/>
       <c r="N57" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B57, $C$2:$C$949, C57, $D$2:$D$949, D57, $E$2:$E$949, E57) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3144,7 +3143,7 @@
         <v>117</v>
       </c>
       <c r="N58" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B58, $C$2:$C$949, C58, $D$2:$D$949, D58, $E$2:$E$949, E58) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3178,7 +3177,7 @@
       </c>
       <c r="J59" s="2"/>
       <c r="N59" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B59, $C$2:$C$949, C59, $D$2:$D$949, D59, $E$2:$E$949, E59) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3217,7 +3216,7 @@
         <v>169</v>
       </c>
       <c r="N60" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B60, $C$2:$C$949, C60, $D$2:$D$949, D60, $E$2:$E$949, E60) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3251,7 +3250,7 @@
       </c>
       <c r="J61" s="2"/>
       <c r="N61" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B61, $C$2:$C$949, C61, $D$2:$D$949, D61, $E$2:$E$949, E61) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3285,7 +3284,7 @@
       </c>
       <c r="J62" s="2"/>
       <c r="N62" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B62, $C$2:$C$949, C62, $D$2:$D$949, D62, $E$2:$E$949, E62) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3319,7 +3318,7 @@
       </c>
       <c r="J63" s="2"/>
       <c r="N63" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B63, $C$2:$C$949, C63, $D$2:$D$949, D63, $E$2:$E$949, E63) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3353,7 +3352,7 @@
       </c>
       <c r="J64" s="2"/>
       <c r="N64" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B64, $C$2:$C$949, C64, $D$2:$D$949, D64, $E$2:$E$949, E64) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3387,7 +3386,7 @@
       </c>
       <c r="J65" s="2"/>
       <c r="N65" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B65, $C$2:$C$949, C65, $D$2:$D$949, D65, $E$2:$E$949, E65) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3421,7 +3420,7 @@
       </c>
       <c r="J66" s="2"/>
       <c r="N66" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B66, $C$2:$C$949, C66, $D$2:$D$949, D66, $E$2:$E$949, E66) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N66:N129" si="1">IF(COUNTIFS( $B$2:$B$949, B66, $C$2:$C$949, C66, $D$2:$D$949, D66, $E$2:$E$949, E66) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -3455,7 +3454,7 @@
       </c>
       <c r="J67" s="2"/>
       <c r="N67" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B67, $C$2:$C$949, C67, $D$2:$D$949, D67, $E$2:$E$949, E67) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3491,7 +3490,7 @@
         <v>41</v>
       </c>
       <c r="N68" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B68, $C$2:$C$949, C68, $D$2:$D$949, D68, $E$2:$E$949, E68) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3525,7 +3524,7 @@
       </c>
       <c r="J69" s="2"/>
       <c r="N69" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B69, $C$2:$C$949, C69, $D$2:$D$949, D69, $E$2:$E$949, E69) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3559,7 +3558,7 @@
       </c>
       <c r="J70" s="2"/>
       <c r="N70" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B70, $C$2:$C$949, C70, $D$2:$D$949, D70, $E$2:$E$949, E70) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3595,7 +3594,7 @@
         <v>41</v>
       </c>
       <c r="N71" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B71, $C$2:$C$949, C71, $D$2:$D$949, D71, $E$2:$E$949, E71) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3629,7 +3628,7 @@
       </c>
       <c r="J72" s="2"/>
       <c r="N72" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B72, $C$2:$C$949, C72, $D$2:$D$949, D72, $E$2:$E$949, E72) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3663,7 +3662,7 @@
       </c>
       <c r="J73" s="2"/>
       <c r="N73" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B73, $C$2:$C$949, C73, $D$2:$D$949, D73, $E$2:$E$949, E73) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3697,7 +3696,7 @@
       </c>
       <c r="J74" s="2"/>
       <c r="N74" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B74, $C$2:$C$949, C74, $D$2:$D$949, D74, $E$2:$E$949, E74) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3731,7 +3730,7 @@
       </c>
       <c r="J75" s="2"/>
       <c r="N75" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B75, $C$2:$C$949, C75, $D$2:$D$949, D75, $E$2:$E$949, E75) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3765,7 +3764,7 @@
       </c>
       <c r="J76" s="2"/>
       <c r="N76" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B76, $C$2:$C$949, C76, $D$2:$D$949, D76, $E$2:$E$949, E76) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3799,7 +3798,7 @@
       </c>
       <c r="J77" s="2"/>
       <c r="N77" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B77, $C$2:$C$949, C77, $D$2:$D$949, D77, $E$2:$E$949, E77) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3836,7 +3835,7 @@
         <v>156</v>
       </c>
       <c r="N78" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B78, $C$2:$C$949, C78, $D$2:$D$949, D78, $E$2:$E$949, E78) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3870,7 +3869,7 @@
       </c>
       <c r="J79" s="2"/>
       <c r="N79" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B79, $C$2:$C$949, C79, $D$2:$D$949, D79, $E$2:$E$949, E79) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3904,7 +3903,7 @@
       </c>
       <c r="J80" s="2"/>
       <c r="N80" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B80, $C$2:$C$949, C80, $D$2:$D$949, D80, $E$2:$E$949, E80) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3938,7 +3937,7 @@
       </c>
       <c r="J81" s="2"/>
       <c r="N81" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B81, $C$2:$C$949, C81, $D$2:$D$949, D81, $E$2:$E$949, E81) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3972,7 +3971,7 @@
       </c>
       <c r="J82" s="2"/>
       <c r="N82" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B82, $C$2:$C$949, C82, $D$2:$D$949, D82, $E$2:$E$949, E82) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4006,7 +4005,7 @@
       </c>
       <c r="J83" s="2"/>
       <c r="N83" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B83, $C$2:$C$949, C83, $D$2:$D$949, D83, $E$2:$E$949, E83) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4040,7 +4039,7 @@
       </c>
       <c r="J84" s="2"/>
       <c r="N84" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B84, $C$2:$C$949, C84, $D$2:$D$949, D84, $E$2:$E$949, E84) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4074,7 +4073,7 @@
       </c>
       <c r="J85" s="2"/>
       <c r="N85" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B85, $C$2:$C$949, C85, $D$2:$D$949, D85, $E$2:$E$949, E85) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4108,7 +4107,7 @@
       </c>
       <c r="J86" s="2"/>
       <c r="N86" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B86, $C$2:$C$949, C86, $D$2:$D$949, D86, $E$2:$E$949, E86) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4142,7 +4141,7 @@
       </c>
       <c r="J87" s="2"/>
       <c r="N87" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B87, $C$2:$C$949, C87, $D$2:$D$949, D87, $E$2:$E$949, E87) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4178,7 +4177,7 @@
         <v>41</v>
       </c>
       <c r="N88" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B88, $C$2:$C$949, C88, $D$2:$D$949, D88, $E$2:$E$949, E88) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4212,7 +4211,7 @@
       </c>
       <c r="J89" s="2"/>
       <c r="N89" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B89, $C$2:$C$949, C89, $D$2:$D$949, D89, $E$2:$E$949, E89) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4246,7 +4245,7 @@
       </c>
       <c r="J90" s="2"/>
       <c r="N90" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B90, $C$2:$C$949, C90, $D$2:$D$949, D90, $E$2:$E$949, E90) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4282,7 +4281,7 @@
         <v>141</v>
       </c>
       <c r="N91" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B91, $C$2:$C$949, C91, $D$2:$D$949, D91, $E$2:$E$949, E91) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4316,7 +4315,7 @@
       </c>
       <c r="J92" s="2"/>
       <c r="N92" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B92, $C$2:$C$949, C92, $D$2:$D$949, D92, $E$2:$E$949, E92) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4350,7 +4349,7 @@
       </c>
       <c r="J93" s="2"/>
       <c r="N93" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B93, $C$2:$C$949, C93, $D$2:$D$949, D93, $E$2:$E$949, E93) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4384,7 +4383,7 @@
       </c>
       <c r="J94" s="2"/>
       <c r="N94" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B94, $C$2:$C$949, C94, $D$2:$D$949, D94, $E$2:$E$949, E94) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4420,7 +4419,7 @@
         <v>41</v>
       </c>
       <c r="N95" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B95, $C$2:$C$949, C95, $D$2:$D$949, D95, $E$2:$E$949, E95) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4454,7 +4453,7 @@
       </c>
       <c r="J96" s="2"/>
       <c r="N96" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B96, $C$2:$C$949, C96, $D$2:$D$949, D96, $E$2:$E$949, E96) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4488,7 +4487,7 @@
       </c>
       <c r="J97" s="2"/>
       <c r="N97" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B97, $C$2:$C$949, C97, $D$2:$D$949, D97, $E$2:$E$949, E97) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4522,7 +4521,7 @@
       </c>
       <c r="J98" s="2"/>
       <c r="N98" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B98, $C$2:$C$949, C98, $D$2:$D$949, D98, $E$2:$E$949, E98) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4556,7 +4555,7 @@
       </c>
       <c r="J99" s="2"/>
       <c r="N99" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B99, $C$2:$C$949, C99, $D$2:$D$949, D99, $E$2:$E$949, E99) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4590,7 +4589,7 @@
       </c>
       <c r="J100" s="2"/>
       <c r="N100" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B100, $C$2:$C$949, C100, $D$2:$D$949, D100, $E$2:$E$949, E100) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4624,7 +4623,7 @@
       </c>
       <c r="J101" s="2"/>
       <c r="N101" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B101, $C$2:$C$949, C101, $D$2:$D$949, D101, $E$2:$E$949, E101) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4658,7 +4657,7 @@
       </c>
       <c r="J102" s="2"/>
       <c r="N102" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B102, $C$2:$C$949, C102, $D$2:$D$949, D102, $E$2:$E$949, E102) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4692,7 +4691,7 @@
       </c>
       <c r="J103" s="2"/>
       <c r="N103" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B103, $C$2:$C$949, C103, $D$2:$D$949, D103, $E$2:$E$949, E103) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4726,7 +4725,7 @@
       </c>
       <c r="J104" s="2"/>
       <c r="N104" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B104, $C$2:$C$949, C104, $D$2:$D$949, D104, $E$2:$E$949, E104) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4760,7 +4759,7 @@
       </c>
       <c r="J105" s="2"/>
       <c r="N105" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B105, $C$2:$C$949, C105, $D$2:$D$949, D105, $E$2:$E$949, E105) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4794,7 +4793,7 @@
       </c>
       <c r="J106" s="2"/>
       <c r="N106" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B106, $C$2:$C$949, C106, $D$2:$D$949, D106, $E$2:$E$949, E106) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4828,7 +4827,7 @@
       </c>
       <c r="J107" s="2"/>
       <c r="N107" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B107, $C$2:$C$949, C107, $D$2:$D$949, D107, $E$2:$E$949, E107) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4862,7 +4861,7 @@
       </c>
       <c r="J108" s="2"/>
       <c r="N108" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B108, $C$2:$C$949, C108, $D$2:$D$949, D108, $E$2:$E$949, E108) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4896,7 +4895,7 @@
       </c>
       <c r="J109" s="2"/>
       <c r="N109" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B109, $C$2:$C$949, C109, $D$2:$D$949, D109, $E$2:$E$949, E109) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4930,7 +4929,7 @@
       </c>
       <c r="J110" s="2"/>
       <c r="N110" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B110, $C$2:$C$949, C110, $D$2:$D$949, D110, $E$2:$E$949, E110) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4964,7 +4963,7 @@
       </c>
       <c r="J111" s="2"/>
       <c r="N111" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B111, $C$2:$C$949, C111, $D$2:$D$949, D111, $E$2:$E$949, E111) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4998,7 +4997,7 @@
       </c>
       <c r="J112" s="2"/>
       <c r="N112" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B112, $C$2:$C$949, C112, $D$2:$D$949, D112, $E$2:$E$949, E112) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5032,7 +5031,7 @@
       </c>
       <c r="J113" s="2"/>
       <c r="N113" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B113, $C$2:$C$949, C113, $D$2:$D$949, D113, $E$2:$E$949, E113) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5068,7 +5067,7 @@
         <v>41</v>
       </c>
       <c r="N114" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B114, $C$2:$C$949, C114, $D$2:$D$949, D114, $E$2:$E$949, E114) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5102,7 +5101,7 @@
       </c>
       <c r="J115" s="2"/>
       <c r="N115" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B115, $C$2:$C$949, C115, $D$2:$D$949, D115, $E$2:$E$949, E115) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5136,7 +5135,7 @@
       </c>
       <c r="J116" s="2"/>
       <c r="N116" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B116, $C$2:$C$949, C116, $D$2:$D$949, D116, $E$2:$E$949, E116) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5170,7 +5169,7 @@
       </c>
       <c r="J117" s="2"/>
       <c r="N117" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B117, $C$2:$C$949, C117, $D$2:$D$949, D117, $E$2:$E$949, E117) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5204,7 +5203,7 @@
       </c>
       <c r="J118" s="2"/>
       <c r="N118" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B118, $C$2:$C$949, C118, $D$2:$D$949, D118, $E$2:$E$949, E118) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5238,7 +5237,7 @@
       </c>
       <c r="J119" s="2"/>
       <c r="N119" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B119, $C$2:$C$949, C119, $D$2:$D$949, D119, $E$2:$E$949, E119) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5272,7 +5271,7 @@
       </c>
       <c r="J120" s="2"/>
       <c r="N120" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B120, $C$2:$C$949, C120, $D$2:$D$949, D120, $E$2:$E$949, E120) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5306,7 +5305,7 @@
       </c>
       <c r="J121" s="2"/>
       <c r="N121" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B121, $C$2:$C$949, C121, $D$2:$D$949, D121, $E$2:$E$949, E121) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5340,7 +5339,7 @@
       </c>
       <c r="J122" s="2"/>
       <c r="N122" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B122, $C$2:$C$949, C122, $D$2:$D$949, D122, $E$2:$E$949, E122) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5374,7 +5373,7 @@
       </c>
       <c r="J123" s="2"/>
       <c r="N123" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B123, $C$2:$C$949, C123, $D$2:$D$949, D123, $E$2:$E$949, E123) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5408,7 +5407,7 @@
       </c>
       <c r="J124" s="2"/>
       <c r="N124" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B124, $C$2:$C$949, C124, $D$2:$D$949, D124, $E$2:$E$949, E124) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5442,7 +5441,7 @@
       </c>
       <c r="J125" s="2"/>
       <c r="N125" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B125, $C$2:$C$949, C125, $D$2:$D$949, D125, $E$2:$E$949, E125) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5478,7 +5477,7 @@
         <v>41</v>
       </c>
       <c r="N126" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B126, $C$2:$C$949, C126, $D$2:$D$949, D126, $E$2:$E$949, E126) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5512,7 +5511,7 @@
       </c>
       <c r="J127" s="2"/>
       <c r="N127" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B127, $C$2:$C$949, C127, $D$2:$D$949, D127, $E$2:$E$949, E127) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5548,7 +5547,7 @@
         <v>55</v>
       </c>
       <c r="N128" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B128, $C$2:$C$949, C128, $D$2:$D$949, D128, $E$2:$E$949, E128) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5582,7 +5581,7 @@
       </c>
       <c r="J129" s="2"/>
       <c r="N129" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B129, $C$2:$C$949, C129, $D$2:$D$949, D129, $E$2:$E$949, E129) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5616,7 +5615,7 @@
       </c>
       <c r="J130" s="2"/>
       <c r="N130" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B130, $C$2:$C$949, C130, $D$2:$D$949, D130, $E$2:$E$949, E130) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N130:N193" si="2">IF(COUNTIFS( $B$2:$B$949, B130, $C$2:$C$949, C130, $D$2:$D$949, D130, $E$2:$E$949, E130) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -5655,7 +5654,7 @@
       <c r="L131"/>
       <c r="M131"/>
       <c r="N131" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B131, $C$2:$C$949, C131, $D$2:$D$949, D131, $E$2:$E$949, E131) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5692,7 +5691,7 @@
       <c r="L132"/>
       <c r="M132"/>
       <c r="N132" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B132, $C$2:$C$949, C132, $D$2:$D$949, D132, $E$2:$E$949, E132) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5729,7 +5728,7 @@
       <c r="L133"/>
       <c r="M133"/>
       <c r="N133" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B133, $C$2:$C$949, C133, $D$2:$D$949, D133, $E$2:$E$949, E133) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5766,11 +5765,11 @@
       <c r="L134"/>
       <c r="M134"/>
       <c r="N134" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B134, $C$2:$C$949, C134, $D$2:$D$949, D134, $E$2:$E$949, E134) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="135" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A135" s="25">
         <v>46252.645138888889</v>
       </c>
@@ -5800,11 +5799,11 @@
       </c>
       <c r="J135" s="15"/>
       <c r="N135" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B135, $C$2:$C$949, C135, $D$2:$D$949, D135, $E$2:$E$949, E135) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="136" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A136" s="13" t="s">
         <v>62</v>
       </c>
@@ -5834,7 +5833,7 @@
       </c>
       <c r="J136" s="15"/>
       <c r="N136" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B136, $C$2:$C$949, C136, $D$2:$D$949, D136, $E$2:$E$949, E136) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5873,11 +5872,11 @@
       <c r="L137"/>
       <c r="M137"/>
       <c r="N137" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B137, $C$2:$C$949, C137, $D$2:$D$949, D137, $E$2:$E$949, E137) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="138" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="25">
         <v>46252.645138888889</v>
       </c>
@@ -5907,11 +5906,11 @@
       </c>
       <c r="J138" s="15"/>
       <c r="N138" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B138, $C$2:$C$949, C138, $D$2:$D$949, D138, $E$2:$E$949, E138) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="139" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A139" s="25">
         <v>46252.645833333336</v>
       </c>
@@ -5941,11 +5940,11 @@
       </c>
       <c r="J139" s="15"/>
       <c r="N139" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B139, $C$2:$C$949, C139, $D$2:$D$949, D139, $E$2:$E$949, E139) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="140" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A140" s="25">
         <v>46253.375</v>
       </c>
@@ -5980,11 +5979,11 @@
         <v>152</v>
       </c>
       <c r="N140" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B140, $C$2:$C$949, C140, $D$2:$D$949, D140, $E$2:$E$949, E140) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="141" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="25">
         <v>46252.645138888889</v>
       </c>
@@ -6014,11 +6013,11 @@
       </c>
       <c r="J141" s="15"/>
       <c r="N141" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B141, $C$2:$C$949, C141, $D$2:$D$949, D141, $E$2:$E$949, E141) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="142" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="4" t="s">
         <v>172</v>
       </c>
@@ -6055,11 +6054,11 @@
       <c r="L142"/>
       <c r="M142"/>
       <c r="N142" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B142, $C$2:$C$949, C142, $D$2:$D$949, D142, $E$2:$E$949, E142) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="143" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="3">
         <v>46254.643043981479</v>
       </c>
@@ -6096,11 +6095,11 @@
       <c r="L143"/>
       <c r="M143"/>
       <c r="N143" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B143, $C$2:$C$949, C143, $D$2:$D$949, D143, $E$2:$E$949, E143) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="144" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A144" s="25">
         <v>46253.604166666664</v>
       </c>
@@ -6135,11 +6134,11 @@
         <v>151</v>
       </c>
       <c r="N144" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B144, $C$2:$C$949, C144, $D$2:$D$949, D144, $E$2:$E$949, E144) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="145" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A145" s="25">
         <v>46253.375</v>
       </c>
@@ -6172,11 +6171,11 @@
         <v>150</v>
       </c>
       <c r="N145" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B145, $C$2:$C$949, C145, $D$2:$D$949, D145, $E$2:$E$949, E145) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="146" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="146" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A146" s="25">
         <v>46252.645833333336</v>
       </c>
@@ -6206,11 +6205,11 @@
       </c>
       <c r="J146" s="15"/>
       <c r="N146" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B146, $C$2:$C$949, C146, $D$2:$D$949, D146, $E$2:$E$949, E146) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="147" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="147" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A147" s="13" t="s">
         <v>62</v>
       </c>
@@ -6240,11 +6239,11 @@
       </c>
       <c r="J147" s="15"/>
       <c r="N147" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B147, $C$2:$C$949, C147, $D$2:$D$949, D147, $E$2:$E$949, E147) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="148" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="148" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A148" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6276,11 +6275,11 @@
         <v>55</v>
       </c>
       <c r="N148" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B148, $C$2:$C$949, C148, $D$2:$D$949, D148, $E$2:$E$949, E148) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="149" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="149" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A149" s="25">
         <v>46252.6875</v>
       </c>
@@ -6310,11 +6309,11 @@
       </c>
       <c r="J149" s="15"/>
       <c r="N149" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B149, $C$2:$C$949, C149, $D$2:$D$949, D149, $E$2:$E$949, E149) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="150" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="150" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A150" s="25">
         <v>46252.6875</v>
       </c>
@@ -6346,11 +6345,11 @@
         <v>55</v>
       </c>
       <c r="N150" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B150, $C$2:$C$949, C150, $D$2:$D$949, D150, $E$2:$E$949, E150) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="151" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="151" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A151" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6380,11 +6379,11 @@
       </c>
       <c r="J151" s="15"/>
       <c r="N151" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B151, $C$2:$C$949, C151, $D$2:$D$949, D151, $E$2:$E$949, E151) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="152" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="152" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A152" s="25">
         <v>46253.522916666669</v>
       </c>
@@ -6419,11 +6418,11 @@
         <v>153</v>
       </c>
       <c r="N152" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B152, $C$2:$C$949, C152, $D$2:$D$949, D152, $E$2:$E$949, E152) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="153" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="153" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A153" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6453,11 +6452,11 @@
       </c>
       <c r="J153" s="15"/>
       <c r="N153" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B153, $C$2:$C$949, C153, $D$2:$D$949, D153, $E$2:$E$949, E153) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="154" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="154" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A154" s="13" t="s">
         <v>62</v>
       </c>
@@ -6489,11 +6488,11 @@
         <v>41</v>
       </c>
       <c r="N154" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B154, $C$2:$C$949, C154, $D$2:$D$949, D154, $E$2:$E$949, E154) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="155" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A155" s="3">
         <v>46254.625937500001</v>
       </c>
@@ -6530,11 +6529,11 @@
       <c r="L155"/>
       <c r="M155"/>
       <c r="N155" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B155, $C$2:$C$949, C155, $D$2:$D$949, D155, $E$2:$E$949, E155) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="156" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="156" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A156" s="25">
         <v>46252.6875</v>
       </c>
@@ -6566,11 +6565,11 @@
         <v>41</v>
       </c>
       <c r="N156" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B156, $C$2:$C$949, C156, $D$2:$D$949, D156, $E$2:$E$949, E156) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="157" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A157" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6602,11 +6601,11 @@
         <v>41</v>
       </c>
       <c r="N157" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B157, $C$2:$C$949, C157, $D$2:$D$949, D157, $E$2:$E$949, E157) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="158" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="25">
         <v>46253.629861111112</v>
       </c>
@@ -6639,11 +6638,11 @@
         <v>144</v>
       </c>
       <c r="N158" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B158, $C$2:$C$949, C158, $D$2:$D$949, D158, $E$2:$E$949, E158) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="159" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="25">
         <v>46252.6875</v>
       </c>
@@ -6673,11 +6672,11 @@
       </c>
       <c r="J159" s="15"/>
       <c r="N159" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B159, $C$2:$C$949, C159, $D$2:$D$949, D159, $E$2:$E$949, E159) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="160" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="25">
         <v>46252.6875</v>
       </c>
@@ -6709,11 +6708,11 @@
         <v>55</v>
       </c>
       <c r="N160" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B160, $C$2:$C$949, C160, $D$2:$D$949, D160, $E$2:$E$949, E160) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="161" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="161" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A161" s="25">
         <v>46252.688194444447</v>
       </c>
@@ -6743,11 +6742,11 @@
       </c>
       <c r="J161" s="15"/>
       <c r="N161" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B161, $C$2:$C$949, C161, $D$2:$D$949, D161, $E$2:$E$949, E161) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="162" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="162" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="25">
         <v>46252.645138888889</v>
       </c>
@@ -6777,11 +6776,11 @@
       </c>
       <c r="J162" s="15"/>
       <c r="N162" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B162, $C$2:$C$949, C162, $D$2:$D$949, D162, $E$2:$E$949, E162) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="163" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="163" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A163" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6811,11 +6810,11 @@
       </c>
       <c r="J163" s="15"/>
       <c r="N163" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B163, $C$2:$C$949, C163, $D$2:$D$949, D163, $E$2:$E$949, E163) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="164" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="164" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A164" s="13" t="s">
         <v>62</v>
       </c>
@@ -6847,11 +6846,11 @@
         <v>41</v>
       </c>
       <c r="N164" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B164, $C$2:$C$949, C164, $D$2:$D$949, D164, $E$2:$E$949, E164) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="165" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="165" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="25">
         <v>46252.6875</v>
       </c>
@@ -6881,11 +6880,11 @@
       </c>
       <c r="J165" s="15"/>
       <c r="N165" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B165, $C$2:$C$949, C165, $D$2:$D$949, D165, $E$2:$E$949, E165) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="166" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="166" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A166" s="25">
         <v>46252.645833333336</v>
       </c>
@@ -6915,11 +6914,11 @@
       </c>
       <c r="J166" s="15"/>
       <c r="N166" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B166, $C$2:$C$949, C166, $D$2:$D$949, D166, $E$2:$E$949, E166) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="167" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="167" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A167" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -6954,11 +6953,11 @@
         <v>155</v>
       </c>
       <c r="N167" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B167, $C$2:$C$949, C167, $D$2:$D$949, D167, $E$2:$E$949, E167) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="168" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="168" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="13" t="s">
         <v>62</v>
       </c>
@@ -6988,11 +6987,11 @@
       </c>
       <c r="J168" s="15"/>
       <c r="N168" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B168, $C$2:$C$949, C168, $D$2:$D$949, D168, $E$2:$E$949, E168) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="169" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="169" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A169" s="25">
         <v>46253.4</v>
       </c>
@@ -7027,11 +7026,11 @@
         <v>147</v>
       </c>
       <c r="N169" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B169, $C$2:$C$949, C169, $D$2:$D$949, D169, $E$2:$E$949, E169) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="170" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="170" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A170" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -7063,11 +7062,11 @@
         <v>41</v>
       </c>
       <c r="N170" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B170, $C$2:$C$949, C170, $D$2:$D$949, D170, $E$2:$E$949, E170) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="171" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="171" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="25">
         <v>46252.6875</v>
       </c>
@@ -7099,11 +7098,11 @@
         <v>55</v>
       </c>
       <c r="N171" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B171, $C$2:$C$949, C171, $D$2:$D$949, D171, $E$2:$E$949, E171) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="172" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="172" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="13" t="s">
         <v>62</v>
       </c>
@@ -7133,11 +7132,11 @@
       </c>
       <c r="J172" s="15"/>
       <c r="N172" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B172, $C$2:$C$949, C172, $D$2:$D$949, D172, $E$2:$E$949, E172) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="173" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="173" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A173" s="25">
         <v>46253.375</v>
       </c>
@@ -7172,11 +7171,11 @@
         <v>154</v>
       </c>
       <c r="N173" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B173, $C$2:$C$949, C173, $D$2:$D$949, D173, $E$2:$E$949, E173) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="174" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="174" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A174" s="13" t="s">
         <v>62</v>
       </c>
@@ -7208,11 +7207,11 @@
         <v>55</v>
       </c>
       <c r="N174" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B174, $C$2:$C$949, C174, $D$2:$D$949, D174, $E$2:$E$949, E174) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="175" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="175" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A175" s="25">
         <v>46253.395138888889</v>
       </c>
@@ -7245,11 +7244,11 @@
         <v>148</v>
       </c>
       <c r="N175" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B175, $C$2:$C$949, C175, $D$2:$D$949, D175, $E$2:$E$949, E175) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="176" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="176" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A176" s="13" t="s">
         <v>62</v>
       </c>
@@ -7281,11 +7280,11 @@
         <v>118</v>
       </c>
       <c r="N176" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B176, $C$2:$C$949, C176, $D$2:$D$949, D176, $E$2:$E$949, E176) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="177" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="177" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -7315,11 +7314,11 @@
       </c>
       <c r="J177" s="15"/>
       <c r="N177" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B177, $C$2:$C$949, C177, $D$2:$D$949, D177, $E$2:$E$949, E177) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="178" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="178" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="25">
         <v>46252.688194444447</v>
       </c>
@@ -7349,11 +7348,11 @@
       </c>
       <c r="J178" s="15"/>
       <c r="N178" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B178, $C$2:$C$949, C178, $D$2:$D$949, D178, $E$2:$E$949, E178) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="179" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="179" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="3">
         <v>46254.375578703701</v>
       </c>
@@ -7390,11 +7389,11 @@
       <c r="L179"/>
       <c r="M179"/>
       <c r="N179" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B179, $C$2:$C$949, C179, $D$2:$D$949, D179, $E$2:$E$949, E179) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="180" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="180" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A180" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -7424,11 +7423,11 @@
       </c>
       <c r="J180" s="15"/>
       <c r="N180" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B180, $C$2:$C$949, C180, $D$2:$D$949, D180, $E$2:$E$949, E180) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="181" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="181" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A181" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -7458,11 +7457,11 @@
       </c>
       <c r="J181" s="15"/>
       <c r="N181" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B181, $C$2:$C$949, C181, $D$2:$D$949, D181, $E$2:$E$949, E181) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="182" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="182" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A182" s="25">
         <v>46252.688194444447</v>
       </c>
@@ -7492,11 +7491,11 @@
       </c>
       <c r="J182" s="15"/>
       <c r="N182" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B182, $C$2:$C$949, C182, $D$2:$D$949, D182, $E$2:$E$949, E182) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="183" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="183" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A183" s="25">
         <v>46252.6875</v>
       </c>
@@ -7528,11 +7527,11 @@
         <v>55</v>
       </c>
       <c r="N183" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B183, $C$2:$C$949, C183, $D$2:$D$949, D183, $E$2:$E$949, E183) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="184" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A184" s="13" t="s">
         <v>62</v>
       </c>
@@ -7562,11 +7561,11 @@
       </c>
       <c r="J184" s="15"/>
       <c r="N184" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B184, $C$2:$C$949, C184, $D$2:$D$949, D184, $E$2:$E$949, E184) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="185" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="185" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A185" s="13" t="s">
         <v>62</v>
       </c>
@@ -7596,11 +7595,11 @@
       </c>
       <c r="J185" s="15"/>
       <c r="N185" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B185, $C$2:$C$949, C185, $D$2:$D$949, D185, $E$2:$E$949, E185) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="186" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="186" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A186" s="13" t="s">
         <v>62</v>
       </c>
@@ -7632,11 +7631,11 @@
         <v>118</v>
       </c>
       <c r="N186" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B186, $C$2:$C$949, C186, $D$2:$D$949, D186, $E$2:$E$949, E186) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="187" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="187" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A187" s="13" t="s">
         <v>62</v>
       </c>
@@ -7666,11 +7665,11 @@
       </c>
       <c r="J187" s="15"/>
       <c r="N187" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B187, $C$2:$C$949, C187, $D$2:$D$949, D187, $E$2:$E$949, E187) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="188" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="188" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A188" s="13" t="s">
         <v>62</v>
       </c>
@@ -7700,11 +7699,11 @@
       </c>
       <c r="J188" s="15"/>
       <c r="N188" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B188, $C$2:$C$949, C188, $D$2:$D$949, D188, $E$2:$E$949, E188) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="189" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="189" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A189" s="13" t="s">
         <v>62</v>
       </c>
@@ -7736,11 +7735,11 @@
         <v>117</v>
       </c>
       <c r="N189" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B189, $C$2:$C$949, C189, $D$2:$D$949, D189, $E$2:$E$949, E189) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="190" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="190" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A190" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -7770,11 +7769,11 @@
       </c>
       <c r="J190" s="15"/>
       <c r="N190" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B190, $C$2:$C$949, C190, $D$2:$D$949, D190, $E$2:$E$949, E190) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="191" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="191" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A191" s="13" t="s">
         <v>62</v>
       </c>
@@ -7804,11 +7803,11 @@
       </c>
       <c r="J191" s="15"/>
       <c r="N191" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B191, $C$2:$C$949, C191, $D$2:$D$949, D191, $E$2:$E$949, E191) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="192" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="192" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A192" s="13" t="s">
         <v>62</v>
       </c>
@@ -7840,11 +7839,11 @@
         <v>118</v>
       </c>
       <c r="N192" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B192, $C$2:$C$949, C192, $D$2:$D$949, D192, $E$2:$E$949, E192) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="193" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="193" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A193" s="25">
         <v>46252.6875</v>
       </c>
@@ -7876,11 +7875,11 @@
         <v>41</v>
       </c>
       <c r="N193" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B193, $C$2:$C$949, C193, $D$2:$D$949, D193, $E$2:$E$949, E193) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="194" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A194" s="25">
         <v>46252.688194444447</v>
       </c>
@@ -7910,11 +7909,11 @@
       </c>
       <c r="J194" s="15"/>
       <c r="N194" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B194, $C$2:$C$949, C194, $D$2:$D$949, D194, $E$2:$E$949, E194) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="195" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" ref="N194:N245" si="3">IF(COUNTIFS( $B$2:$B$949, B194, $C$2:$C$949, C194, $D$2:$D$949, D194, $E$2:$E$949, E194) &gt; 1, "Duplicate", "Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="195" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A195" s="13" t="s">
         <v>62</v>
       </c>
@@ -7946,11 +7945,11 @@
         <v>118</v>
       </c>
       <c r="N195" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B195, $C$2:$C$949, C195, $D$2:$D$949, D195, $E$2:$E$949, E195) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="196" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A196" s="13" t="s">
         <v>62</v>
       </c>
@@ -7982,11 +7981,11 @@
         <v>41</v>
       </c>
       <c r="N196" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B196, $C$2:$C$949, C196, $D$2:$D$949, D196, $E$2:$E$949, E196) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="197" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="197" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A197" s="25">
         <v>46253.605555555558</v>
       </c>
@@ -8019,11 +8018,11 @@
         <v>145</v>
       </c>
       <c r="N197" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B197, $C$2:$C$949, C197, $D$2:$D$949, D197, $E$2:$E$949, E197) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="198" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="198" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A198" s="13" t="s">
         <v>62</v>
       </c>
@@ -8053,11 +8052,11 @@
       </c>
       <c r="J198" s="15"/>
       <c r="N198" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B198, $C$2:$C$949, C198, $D$2:$D$949, D198, $E$2:$E$949, E198) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="199" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="199" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A199" s="13" t="s">
         <v>62</v>
       </c>
@@ -8087,11 +8086,11 @@
       </c>
       <c r="J199" s="15"/>
       <c r="N199" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B199, $C$2:$C$949, C199, $D$2:$D$949, D199, $E$2:$E$949, E199) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="200" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="200" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A200" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -8121,11 +8120,11 @@
       </c>
       <c r="J200" s="15"/>
       <c r="N200" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B200, $C$2:$C$949, C200, $D$2:$D$949, D200, $E$2:$E$949, E200) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="201" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="201" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A201" s="13" t="s">
         <v>62</v>
       </c>
@@ -8155,11 +8154,11 @@
       </c>
       <c r="J201" s="15"/>
       <c r="N201" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B201, $C$2:$C$949, C201, $D$2:$D$949, D201, $E$2:$E$949, E201) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="202" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="202" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A202" s="25">
         <v>46252.688194444447</v>
       </c>
@@ -8189,11 +8188,11 @@
       </c>
       <c r="J202" s="15"/>
       <c r="N202" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B202, $C$2:$C$949, C202, $D$2:$D$949, D202, $E$2:$E$949, E202) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="203" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="203" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A203" s="13" t="s">
         <v>62</v>
       </c>
@@ -8225,11 +8224,11 @@
         <v>117</v>
       </c>
       <c r="N203" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B203, $C$2:$C$949, C203, $D$2:$D$949, D203, $E$2:$E$949, E203) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="204" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="204" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A204" s="13" t="s">
         <v>62</v>
       </c>
@@ -8259,11 +8258,11 @@
       </c>
       <c r="J204" s="15"/>
       <c r="N204" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B204, $C$2:$C$949, C204, $D$2:$D$949, D204, $E$2:$E$949, E204) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="205" spans="1:14" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="205" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A205" s="13" t="s">
         <v>62</v>
       </c>
@@ -8293,11 +8292,11 @@
       </c>
       <c r="J205" s="15"/>
       <c r="N205" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B205, $C$2:$C$949, C205, $D$2:$D$949, D205, $E$2:$E$949, E205) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="206" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="206" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="13" t="s">
         <v>62</v>
       </c>
@@ -8327,11 +8326,11 @@
       </c>
       <c r="J206" s="15"/>
       <c r="N206" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B206, $C$2:$C$949, C206, $D$2:$D$949, D206, $E$2:$E$949, E206) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="207" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="207" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A207" s="25">
         <v>46253.375</v>
       </c>
@@ -8364,11 +8363,11 @@
         <v>149</v>
       </c>
       <c r="N207" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B207, $C$2:$C$949, C207, $D$2:$D$949, D207, $E$2:$E$949, E207) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="208" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="208" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A208" s="13" t="s">
         <v>62</v>
       </c>
@@ -8398,11 +8397,11 @@
       </c>
       <c r="J208" s="15"/>
       <c r="N208" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B208, $C$2:$C$949, C208, $D$2:$D$949, D208, $E$2:$E$949, E208) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="209" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="209" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A209" s="13" t="s">
         <v>62</v>
       </c>
@@ -8432,11 +8431,11 @@
       </c>
       <c r="J209" s="15"/>
       <c r="N209" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B209, $C$2:$C$949, C209, $D$2:$D$949, D209, $E$2:$E$949, E209) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="210" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="210" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A210" s="13" t="s">
         <v>62</v>
       </c>
@@ -8466,11 +8465,11 @@
       </c>
       <c r="J210" s="15"/>
       <c r="N210" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B210, $C$2:$C$949, C210, $D$2:$D$949, D210, $E$2:$E$949, E210) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="211" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="211" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A211" s="25">
         <v>46252.6875</v>
       </c>
@@ -8502,11 +8501,11 @@
         <v>41</v>
       </c>
       <c r="N211" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B211, $C$2:$C$949, C211, $D$2:$D$949, D211, $E$2:$E$949, E211) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="212" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="212" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A212" s="13" t="s">
         <v>62</v>
       </c>
@@ -8536,11 +8535,11 @@
       </c>
       <c r="J212" s="15"/>
       <c r="N212" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B212, $C$2:$C$949, C212, $D$2:$D$949, D212, $E$2:$E$949, E212) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="213" spans="1:14" ht="16.2" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="213" spans="1:14" ht="16.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A213" s="13" t="s">
         <v>62</v>
       </c>
@@ -8570,11 +8569,11 @@
       </c>
       <c r="J213" s="15"/>
       <c r="N213" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B213, $C$2:$C$949, C213, $D$2:$D$949, D213, $E$2:$E$949, E213) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="214" spans="1:14" ht="40.799999999999997" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="214" spans="1:14" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A214" s="13" t="s">
         <v>62</v>
       </c>
@@ -8604,11 +8603,11 @@
       </c>
       <c r="J214" s="15"/>
       <c r="N214" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B214, $C$2:$C$949, C214, $D$2:$D$949, D214, $E$2:$E$949, E214) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="215" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="215" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A215" s="13" t="s">
         <v>62</v>
       </c>
@@ -8638,11 +8637,11 @@
       </c>
       <c r="J215" s="15"/>
       <c r="N215" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B215, $C$2:$C$949, C215, $D$2:$D$949, D215, $E$2:$E$949, E215) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="216" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="216" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A216" s="13" t="s">
         <v>62</v>
       </c>
@@ -8672,11 +8671,11 @@
       </c>
       <c r="J216" s="15"/>
       <c r="N216" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B216, $C$2:$C$949, C216, $D$2:$D$949, D216, $E$2:$E$949, E216) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="217" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="217" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A217" s="13" t="s">
         <v>62</v>
       </c>
@@ -8706,11 +8705,11 @@
       </c>
       <c r="J217" s="15"/>
       <c r="N217" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B217, $C$2:$C$949, C217, $D$2:$D$949, D217, $E$2:$E$949, E217) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="218" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="218" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A218" s="13" t="s">
         <v>62</v>
       </c>
@@ -8742,11 +8741,11 @@
         <v>41</v>
       </c>
       <c r="N218" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B218, $C$2:$C$949, C218, $D$2:$D$949, D218, $E$2:$E$949, E218) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="219" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="219" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A219" s="13" t="s">
         <v>62</v>
       </c>
@@ -8776,11 +8775,11 @@
       </c>
       <c r="J219" s="15"/>
       <c r="N219" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B219, $C$2:$C$949, C219, $D$2:$D$949, D219, $E$2:$E$949, E219) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="220" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="220" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A220" s="13" t="s">
         <v>62</v>
       </c>
@@ -8810,11 +8809,11 @@
       </c>
       <c r="J220" s="15"/>
       <c r="N220" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B220, $C$2:$C$949, C220, $D$2:$D$949, D220, $E$2:$E$949, E220) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="221" spans="1:14" ht="27.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="221" spans="1:14" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A221" s="13" t="s">
         <v>62</v>
       </c>
@@ -8844,11 +8843,11 @@
       </c>
       <c r="J221" s="15"/>
       <c r="N221" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B221, $C$2:$C$949, C221, $D$2:$D$949, D221, $E$2:$E$949, E221) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="222" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="222" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A222" s="13" t="s">
         <v>62</v>
       </c>
@@ -8878,11 +8877,11 @@
       </c>
       <c r="J222" s="15"/>
       <c r="N222" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B222, $C$2:$C$949, C222, $D$2:$D$949, D222, $E$2:$E$949, E222) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="223" spans="1:14" ht="15.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="223" spans="1:14" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A223" s="13" t="s">
         <v>62</v>
       </c>
@@ -8912,11 +8911,11 @@
       </c>
       <c r="J223" s="15"/>
       <c r="N223" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B223, $C$2:$C$949, C223, $D$2:$D$949, D223, $E$2:$E$949, E223) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="224" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="224" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A224" s="25">
         <v>46252.635416666664</v>
       </c>
@@ -8948,11 +8947,11 @@
         <v>55</v>
       </c>
       <c r="N224" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B224, $C$2:$C$949, C224, $D$2:$D$949, D224, $E$2:$E$949, E224) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="225" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="225" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A225" s="13" t="s">
         <v>62</v>
       </c>
@@ -8984,11 +8983,11 @@
         <v>118</v>
       </c>
       <c r="N225" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B225, $C$2:$C$949, C225, $D$2:$D$949, D225, $E$2:$E$949, E225) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="226" spans="1:14" ht="15.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="226" spans="1:14" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A226" s="13" t="s">
         <v>62</v>
       </c>
@@ -9018,11 +9017,11 @@
       </c>
       <c r="J226" s="15"/>
       <c r="N226" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B226, $C$2:$C$949, C226, $D$2:$D$949, D226, $E$2:$E$949, E226) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="227" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="227" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A227" s="13" t="s">
         <v>62</v>
       </c>
@@ -9052,11 +9051,11 @@
       </c>
       <c r="J227" s="15"/>
       <c r="N227" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B227, $C$2:$C$949, C227, $D$2:$D$949, D227, $E$2:$E$949, E227) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="228" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="228" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A228" s="13" t="s">
         <v>62</v>
       </c>
@@ -9088,11 +9087,11 @@
         <v>118</v>
       </c>
       <c r="N228" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B228, $C$2:$C$949, C228, $D$2:$D$949, D228, $E$2:$E$949, E228) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="229" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="229" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A229" s="13" t="s">
         <v>62</v>
       </c>
@@ -9122,11 +9121,11 @@
       </c>
       <c r="J229" s="15"/>
       <c r="N229" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B229, $C$2:$C$949, C229, $D$2:$D$949, D229, $E$2:$E$949, E229) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="230" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="230" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A230" s="13" t="s">
         <v>62</v>
       </c>
@@ -9156,11 +9155,11 @@
       </c>
       <c r="J230" s="15"/>
       <c r="N230" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B230, $C$2:$C$949, C230, $D$2:$D$949, D230, $E$2:$E$949, E230) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="231" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="231" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A231" s="13" t="s">
         <v>62</v>
       </c>
@@ -9190,11 +9189,11 @@
       </c>
       <c r="J231" s="15"/>
       <c r="N231" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B231, $C$2:$C$949, C231, $D$2:$D$949, D231, $E$2:$E$949, E231) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="232" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="232" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A232" s="13" t="s">
         <v>62</v>
       </c>
@@ -9224,11 +9223,11 @@
       </c>
       <c r="J232" s="15"/>
       <c r="N232" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B232, $C$2:$C$949, C232, $D$2:$D$949, D232, $E$2:$E$949, E232) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="233" spans="1:14" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="233" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A233" s="25">
         <v>46252.6875</v>
       </c>
@@ -9260,11 +9259,11 @@
         <v>118</v>
       </c>
       <c r="N233" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B233, $C$2:$C$949, C233, $D$2:$D$949, D233, $E$2:$E$949, E233) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="234" spans="1:14" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="234" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A234" s="13" t="s">
         <v>62</v>
       </c>
@@ -9294,11 +9293,11 @@
       </c>
       <c r="J234" s="15"/>
       <c r="N234" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B234, $C$2:$C$949, C234, $D$2:$D$949, D234, $E$2:$E$949, E234) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="235" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="235" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A235" s="13" t="s">
         <v>62</v>
       </c>
@@ -9330,11 +9329,11 @@
         <v>118</v>
       </c>
       <c r="N235" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B235, $C$2:$C$949, C235, $D$2:$D$949, D235, $E$2:$E$949, E235) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="236" spans="1:14" ht="14.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="236" spans="1:14" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A236" s="13" t="s">
         <v>62</v>
       </c>
@@ -9364,11 +9363,11 @@
       </c>
       <c r="J236" s="15"/>
       <c r="N236" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B236, $C$2:$C$949, C236, $D$2:$D$949, D236, $E$2:$E$949, E236) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="237" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="237" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A237" s="13" t="s">
         <v>62</v>
       </c>
@@ -9403,11 +9402,11 @@
       <c r="L237" s="18"/>
       <c r="M237" s="18"/>
       <c r="N237" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B237, $C$2:$C$949, C237, $D$2:$D$949, D237, $E$2:$E$949, E237) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="238" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="238" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A238" s="14" t="s">
         <v>62</v>
       </c>
@@ -9440,11 +9439,11 @@
       <c r="L238" s="18"/>
       <c r="M238" s="18"/>
       <c r="N238" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B238, $C$2:$C$949, C238, $D$2:$D$949, D238, $E$2:$E$949, E238) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="239" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A239" s="13" t="s">
         <v>62</v>
       </c>
@@ -9477,11 +9476,11 @@
       <c r="L239" s="18"/>
       <c r="M239" s="18"/>
       <c r="N239" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B239, $C$2:$C$949, C239, $D$2:$D$949, D239, $E$2:$E$949, E239) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="240" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="240" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A240" s="13" t="s">
         <v>62</v>
       </c>
@@ -9514,11 +9513,11 @@
       <c r="L240" s="18"/>
       <c r="M240" s="18"/>
       <c r="N240" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B240, $C$2:$C$949, C240, $D$2:$D$949, D240, $E$2:$E$949, E240) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="241" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="241" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A241" s="13" t="s">
         <v>62</v>
       </c>
@@ -9551,11 +9550,11 @@
       <c r="L241" s="18"/>
       <c r="M241" s="18"/>
       <c r="N241" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B241, $C$2:$C$949, C241, $D$2:$D$949, D241, $E$2:$E$949, E241) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="242" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="242" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A242" s="13" t="s">
         <v>62</v>
       </c>
@@ -9590,11 +9589,11 @@
       <c r="L242" s="18"/>
       <c r="M242" s="18"/>
       <c r="N242" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B242, $C$2:$C$949, C242, $D$2:$D$949, D242, $E$2:$E$949, E242) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="243" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="243" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A243" s="13" t="s">
         <v>62</v>
       </c>
@@ -9627,11 +9626,11 @@
       <c r="L243" s="18"/>
       <c r="M243" s="18"/>
       <c r="N243" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B243, $C$2:$C$949, C243, $D$2:$D$949, D243, $E$2:$E$949, E243) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="244" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="244" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A244" s="25">
         <v>46251.506249999999</v>
       </c>
@@ -9664,11 +9663,11 @@
       <c r="L244" s="18"/>
       <c r="M244" s="18"/>
       <c r="N244" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B244, $C$2:$C$949, C244, $D$2:$D$949, D244, $E$2:$E$949, E244) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-    </row>
-    <row r="245" spans="1:14" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="3"/>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="245" spans="1:14" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A245" s="13" t="s">
         <v>62</v>
       </c>
@@ -9701,21 +9700,11 @@
       <c r="L245" s="18"/>
       <c r="M245" s="18"/>
       <c r="N245" s="18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$949, B245, $C$2:$C$949, C245, $D$2:$D$949, D245, $E$2:$E$949, E245) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N245">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="B"/>
-      </filters>
-    </filterColumn>
-    <sortState ref="A2:N140">
-      <sortCondition descending="1" ref="F1:F248"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>